<commit_message>
New reports priced at the October 22 close
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR3LbNEqqh1NJpsKSu2JUT
</commit_message>
<xml_diff>
--- a/data/models/asml.xlsx
+++ b/data/models/asml.xlsx
@@ -1021,7 +1021,7 @@
         <v>18</v>
       </c>
       <c r="C17" s="18" t="n">
-        <v>1558.26</v>
+        <v>1560.54</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="C18" s="19" t="n">
         <f aca="false">C16/C17-1</f>
-        <v>-0.303960976270837</v>
+        <v>-0.304977912058515</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>